<commit_message>
Update parliament data - 2026-03-31
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -416,15 +416,57 @@
     <t xml:space="preserve">Politica internazionale|Politica di sicurezza|Energia</t>
   </si>
   <si>
+    <t xml:space="preserve">26.7151</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feller Olivier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EJPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nach den Geldautomaten: Werden die Unternehmen die nächsten Ziele sein?  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Après les bancomats, les entreprises seront-elles les prochaines cibles ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;- Après les explosions répétées de bancomats en Suisse, le braquage d’une usine localisée à Courchavon le 5 mars 2026 au cours duquel les auteurs ont également mis le feu à des véhicules accolés au bâtiment, marque-t-il une nouvelle escalade de la criminalité&amp;nbsp;?&amp;nbsp;&lt;br&gt;- La Confédération traitera-t-elle les braquages d’entreprises de la même manière que les explosions de bancomats&amp;nbsp;?&amp;nbsp;&lt;br&gt;- Par exemple en créant un groupe d’experts&amp;nbsp;?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;- Ist der Raubüberfall auf eine Fabrik in Courchavon am 5.&amp;nbsp;März&amp;nbsp;2026, bei dem die Täter auch zwei neben dem Gebäude geparkte Fahrzeuge in Brand setzten, nach den wiederholten Geldautomat-Sprengungen in der Schweiz ein Zeichen für eine erneute Eskalation der Kriminalität?&amp;nbsp;&lt;br&gt;- Wird der Bund Raubüberfälle auf Unternehmen genauso handhaben wie Sprengungen von Geldautomaten?&amp;nbsp;&lt;br&gt;- Zum Beispiel, indem er eine Expertengruppe einberuft?&amp;nbsp;&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267151</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267151</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conseil fédéral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wirtschaft|Strafrecht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Économie|Droit pénal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Economia|Diritto penale</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.3069</t>
   </si>
   <si>
     <t xml:space="preserve">Sollberger Sandra</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-09</t>
-  </si>
-  <si>
     <t xml:space="preserve">Verkehrssicherheit stärken mit Projekten entlang der N18</t>
   </si>
   <si>
@@ -441,48 +483,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263069</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.7151</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feller Olivier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PLR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EJPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nach den Geldautomaten: Werden die Unternehmen die nächsten Ziele sein?  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Après les bancomats, les entreprises seront-elles les prochaines cibles ? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;- Après les explosions répétées de bancomats en Suisse, le braquage d’une usine localisée à Courchavon le 5 mars 2026 au cours duquel les auteurs ont également mis le feu à des véhicules accolés au bâtiment, marque-t-il une nouvelle escalade de la criminalité&amp;nbsp;?&amp;nbsp;&lt;br&gt;- La Confédération traitera-t-elle les braquages d’entreprises de la même manière que les explosions de bancomats&amp;nbsp;?&amp;nbsp;&lt;br&gt;- Par exemple en créant un groupe d’experts&amp;nbsp;?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;- Ist der Raubüberfall auf eine Fabrik in Courchavon am 5.&amp;nbsp;März&amp;nbsp;2026, bei dem die Täter auch zwei neben dem Gebäude geparkte Fahrzeuge in Brand setzten, nach den wiederholten Geldautomat-Sprengungen in der Schweiz ein Zeichen für eine erneute Eskalation der Kriminalität?&amp;nbsp;&lt;br&gt;- Wird der Bund Raubüberfälle auf Unternehmen genauso handhaben wie Sprengungen von Geldautomaten?&amp;nbsp;&lt;br&gt;- Zum Beispiel, indem er eine Expertengruppe einberuft?&amp;nbsp;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267151</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267151</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conseil fédéral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wirtschaft|Strafrecht</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Économie|Droit pénal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Economia|Diritto penale</t>
   </si>
   <si>
     <t xml:space="preserve">26.030</t>
@@ -5590,62 +5590,62 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>20263069</v>
+        <v>20267151</v>
       </c>
       <c r="B12" t="s">
         <v>134</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>120</v>
       </c>
       <c r="D12" t="s">
         <v>135</v>
       </c>
       <c r="E12" t="s">
-        <v>54</v>
+        <v>136</v>
       </c>
       <c r="F12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G12" t="s">
         <v>25</v>
       </c>
-      <c r="H12"/>
+      <c r="H12" t="s">
+        <v>138</v>
+      </c>
       <c r="I12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="J12" t="s">
-        <v>138</v>
-      </c>
-      <c r="K12" t="s">
-        <v>28</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="K12"/>
       <c r="L12" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="M12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="N12" t="s">
-        <v>30</v>
+        <v>128</v>
       </c>
       <c r="O12" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="P12" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="Q12" t="s">
-        <v>33</v>
+        <v>145</v>
       </c>
       <c r="R12" t="s">
-        <v>59</v>
+        <v>146</v>
       </c>
       <c r="S12" t="s">
-        <v>60</v>
+        <v>147</v>
       </c>
       <c r="T12" t="s">
-        <v>61</v>
+        <v>148</v>
       </c>
       <c r="U12" t="s">
         <v>37</v>
@@ -5653,62 +5653,62 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>20267151</v>
+        <v>20263069</v>
       </c>
       <c r="B13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C13" t="s">
-        <v>120</v>
+        <v>52</v>
       </c>
       <c r="D13" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="E13" t="s">
-        <v>145</v>
+        <v>54</v>
       </c>
       <c r="F13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G13" t="s">
         <v>25</v>
       </c>
-      <c r="H13" t="s">
-        <v>146</v>
-      </c>
+      <c r="H13"/>
       <c r="I13" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="J13" t="s">
-        <v>148</v>
-      </c>
-      <c r="K13"/>
+        <v>152</v>
+      </c>
+      <c r="K13" t="s">
+        <v>28</v>
+      </c>
       <c r="L13" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="M13" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="N13" t="s">
-        <v>128</v>
+        <v>30</v>
       </c>
       <c r="O13" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="P13" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="Q13" t="s">
-        <v>153</v>
+        <v>33</v>
       </c>
       <c r="R13" t="s">
-        <v>154</v>
+        <v>59</v>
       </c>
       <c r="S13" t="s">
-        <v>155</v>
+        <v>60</v>
       </c>
       <c r="T13" t="s">
-        <v>156</v>
+        <v>61</v>
       </c>
       <c r="U13" t="s">
         <v>37</v>
@@ -5731,7 +5731,7 @@
       </c>
       <c r="G14"/>
       <c r="H14" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I14" t="s">
         <v>160</v>
@@ -5918,7 +5918,7 @@
         <v>41</v>
       </c>
       <c r="H17" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I17" t="s">
         <v>198</v>
@@ -6075,7 +6075,7 @@
         <v>233</v>
       </c>
       <c r="Q19" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R19" t="s">
         <v>234</v>
@@ -6178,7 +6178,7 @@
         <v>41</v>
       </c>
       <c r="H21" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I21" t="s">
         <v>251</v>
@@ -6270,7 +6270,7 @@
         <v>271</v>
       </c>
       <c r="Q22" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R22" t="s">
         <v>272</v>
@@ -6335,7 +6335,7 @@
         <v>283</v>
       </c>
       <c r="Q23" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R23" t="s">
         <v>193</v>
@@ -6501,7 +6501,7 @@
         <v>25</v>
       </c>
       <c r="H26" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I26" t="s">
         <v>309</v>
@@ -7044,7 +7044,7 @@
         <v>399</v>
       </c>
       <c r="Q34" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R34" t="s">
         <v>400</v>
@@ -7203,7 +7203,7 @@
         <v>431</v>
       </c>
       <c r="E37" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="F37" t="s">
         <v>432</v>
@@ -7365,7 +7365,7 @@
         <v>459</v>
       </c>
       <c r="Q39" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R39" t="s">
         <v>460</v>
@@ -7403,7 +7403,7 @@
         <v>25</v>
       </c>
       <c r="H40" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I40" t="s">
         <v>465</v>
@@ -7676,7 +7676,7 @@
         <v>518</v>
       </c>
       <c r="Q44" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R44" t="s">
         <v>519</v>
@@ -7934,7 +7934,7 @@
         <v>567</v>
       </c>
       <c r="Q48" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R48" t="s">
         <v>568</v>
@@ -8156,7 +8156,7 @@
         <v>605</v>
       </c>
       <c r="E52" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="F52" t="s">
         <v>606</v>
@@ -8322,7 +8322,7 @@
         <v>634</v>
       </c>
       <c r="Q54" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R54" t="s">
         <v>635</v>
@@ -8645,7 +8645,7 @@
         <v>692</v>
       </c>
       <c r="Q59" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R59" t="s">
         <v>440</v>
@@ -8840,7 +8840,7 @@
         <v>722</v>
       </c>
       <c r="Q62" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R62" t="s">
         <v>723</v>
@@ -8994,7 +8994,7 @@
       </c>
       <c r="G65"/>
       <c r="H65" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I65" t="s">
         <v>502</v>
@@ -9051,7 +9051,7 @@
         <v>41</v>
       </c>
       <c r="H66" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I66" t="s">
         <v>760</v>
@@ -9273,7 +9273,7 @@
         <v>802</v>
       </c>
       <c r="Q69" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R69" t="s">
         <v>803</v>
@@ -9376,7 +9376,7 @@
         <v>25</v>
       </c>
       <c r="H71" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I71" t="s">
         <v>819</v>
@@ -9403,7 +9403,7 @@
         <v>825</v>
       </c>
       <c r="Q71" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R71" t="s">
         <v>826</v>
@@ -9598,7 +9598,7 @@
         <v>861</v>
       </c>
       <c r="Q74" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R74" t="s">
         <v>862</v>
@@ -9756,7 +9756,7 @@
         <v>25</v>
       </c>
       <c r="H77" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I77" t="s">
         <v>885</v>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="G79"/>
       <c r="H79" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I79" t="s">
         <v>905</v>
@@ -10086,7 +10086,7 @@
         <v>944</v>
       </c>
       <c r="Q82" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R82" t="s">
         <v>945</v>
@@ -10151,7 +10151,7 @@
         <v>957</v>
       </c>
       <c r="Q83" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R83" t="s">
         <v>958</v>
@@ -10411,7 +10411,7 @@
         <v>1000</v>
       </c>
       <c r="Q87" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R87" t="s">
         <v>304</v>
@@ -10449,7 +10449,7 @@
         <v>25</v>
       </c>
       <c r="H88" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I88" t="s">
         <v>1003</v>
@@ -10640,7 +10640,7 @@
         <v>25</v>
       </c>
       <c r="H91" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I91" t="s">
         <v>1027</v>
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="H92" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I92" t="s">
         <v>1027</v>
@@ -10766,7 +10766,7 @@
         <v>25</v>
       </c>
       <c r="H93" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I93" t="s">
         <v>1027</v>
@@ -11051,7 +11051,7 @@
         <v>1084</v>
       </c>
       <c r="Q97" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R97" t="s">
         <v>1085</v>
@@ -11177,7 +11177,7 @@
         <v>1107</v>
       </c>
       <c r="Q99" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R99" t="s">
         <v>1108</v>
@@ -11242,7 +11242,7 @@
         <v>1119</v>
       </c>
       <c r="Q100" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R100" t="s">
         <v>1120</v>
@@ -11372,7 +11372,7 @@
         <v>1139</v>
       </c>
       <c r="Q102" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R102" t="s">
         <v>1140</v>
@@ -11790,7 +11790,7 @@
       </c>
       <c r="G109"/>
       <c r="H109" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I109" t="s">
         <v>1203</v>
@@ -11847,7 +11847,7 @@
       </c>
       <c r="G110"/>
       <c r="H110" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I110" t="s">
         <v>1214</v>
@@ -12134,7 +12134,7 @@
         <v>1266</v>
       </c>
       <c r="Q114" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R114" t="s">
         <v>1097</v>
@@ -12264,7 +12264,7 @@
         <v>1288</v>
       </c>
       <c r="Q116" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R116" t="s">
         <v>1289</v>
@@ -12459,7 +12459,7 @@
         <v>1321</v>
       </c>
       <c r="Q119" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R119" t="s">
         <v>1322</v>
@@ -12524,7 +12524,7 @@
         <v>1334</v>
       </c>
       <c r="Q120" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R120" t="s">
         <v>646</v>
@@ -12973,7 +12973,7 @@
         <v>1400</v>
       </c>
       <c r="Q127" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R127" t="s">
         <v>1401</v>
@@ -13038,7 +13038,7 @@
         <v>1411</v>
       </c>
       <c r="Q128" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R128" t="s">
         <v>1412</v>
@@ -13103,7 +13103,7 @@
         <v>1424</v>
       </c>
       <c r="Q129" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R129" t="s">
         <v>1425</v>
@@ -13168,7 +13168,7 @@
         <v>1430</v>
       </c>
       <c r="Q130" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R130" t="s">
         <v>1431</v>
@@ -13197,7 +13197,7 @@
         <v>1435</v>
       </c>
       <c r="E131" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="F131" t="s">
         <v>1436</v>
@@ -13233,7 +13233,7 @@
         <v>1443</v>
       </c>
       <c r="Q131" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R131" t="s">
         <v>440</v>
@@ -13426,7 +13426,7 @@
         <v>1475</v>
       </c>
       <c r="Q134" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R134" t="s">
         <v>1465</v>
@@ -13518,7 +13518,7 @@
         <v>1484</v>
       </c>
       <c r="E136" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="F136" t="s">
         <v>1485</v>
@@ -13615,7 +13615,7 @@
         <v>1499</v>
       </c>
       <c r="Q137" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="R137" t="s">
         <v>1500</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-04-04
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -263,15 +263,48 @@
     <t xml:space="preserve">Trasporti</t>
   </si>
   <si>
+    <t xml:space="preserve">26.3323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brenzikofer Florence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERT-E-S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WBF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hochschulfinanzierung mit alternativen Finanzierungsmodellen sichern</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;In diesem Zusammenhang stellen sich folgende Fragen:&lt;/p&gt;&lt;ol&gt;&lt;li&gt;Welche der aufgeführten Varianten erachtet der Bundesrat als rechtlich umsetzbar, finanzpolitisch nachhaltig und föderal ausgewogen und wie begründet er seine Einschätzung?&lt;/li&gt;&lt;li&gt;Welche Kombination von Instrumenten erscheint geeignet, um die langfristige Stabilität der Hochschulfinanzierung sicherzustellen?&lt;/li&gt;&lt;li&gt;Sieht der Bundesrat im Rahmen des nationalen Finanzausgleichs (NFA) die Möglichkeit, die Unterdeckung zu den Vollkosten für einen Studierenden aus einem Nichthochschulkanton zu einem vereinbarten Teil zur Verrechnung zu bringen? Und zu welchem Teil?&lt;/li&gt;&lt;li&gt;Sieht der Bundesrat in einer Fondslösung, gespiesen aus allfälligen Ausschüttungsüberschüssen der&amp;nbsp;Schweizerischen Nationalbank, unter Wahrung der Unabhängigkeit der Nationalbank und der geltenden Ausschüttungsmechanismen, einen möglichen Weg, den es sich zu prüfen lohnt?&amp;nbsp;Falls nein, wieso nicht?&lt;/li&gt;&lt;li&gt;Könnte die Schaffung eines zweckgebundenen Ausgleichs- und Stabilitätsfonds zur Abfederung finanzpolitischer und struktureller Schwankungen in der Hochschulfinanzierung ausgleichend wirken?&lt;/li&gt;&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanzwesen|Bildung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finances|Éducation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanze|Formazione</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.3228</t>
   </si>
   <si>
     <t xml:space="preserve">Tuosto Brenda</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-19</t>
-  </si>
-  <si>
     <t xml:space="preserve">Planification ferroviaire : Le Conseil fédéral peut-il ignorer les mandats du Parlement ?</t>
   </si>
   <si>
@@ -293,39 +326,6 @@
     <t xml:space="preserve">Trasporti|Pianificazione territoriale e alloggi</t>
   </si>
   <si>
-    <t xml:space="preserve">26.3323</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brenzikofer Florence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VERT-E-S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WBF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hochschulfinanzierung mit alternativen Finanzierungsmodellen sichern</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;In diesem Zusammenhang stellen sich folgende Fragen:&lt;/p&gt;&lt;ol&gt;&lt;li&gt;Welche der aufgeführten Varianten erachtet der Bundesrat als rechtlich umsetzbar, finanzpolitisch nachhaltig und föderal ausgewogen und wie begründet er seine Einschätzung?&lt;/li&gt;&lt;li&gt;Welche Kombination von Instrumenten erscheint geeignet, um die langfristige Stabilität der Hochschulfinanzierung sicherzustellen?&lt;/li&gt;&lt;li&gt;Sieht der Bundesrat im Rahmen des nationalen Finanzausgleichs (NFA) die Möglichkeit, die Unterdeckung zu den Vollkosten für einen Studierenden aus einem Nichthochschulkanton zu einem vereinbarten Teil zur Verrechnung zu bringen? Und zu welchem Teil?&lt;/li&gt;&lt;li&gt;Sieht der Bundesrat in einer Fondslösung, gespiesen aus allfälligen Ausschüttungsüberschüssen der&amp;nbsp;Schweizerischen Nationalbank, unter Wahrung der Unabhängigkeit der Nationalbank und der geltenden Ausschüttungsmechanismen, einen möglichen Weg, den es sich zu prüfen lohnt?&amp;nbsp;Falls nein, wieso nicht?&lt;/li&gt;&lt;li&gt;Könnte die Schaffung eines zweckgebundenen Ausgleichs- und Stabilitätsfonds zur Abfederung finanzpolitischer und struktureller Schwankungen in der Hochschulfinanzierung ausgleichend wirken?&lt;/li&gt;&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263323</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263323</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanzwesen|Bildung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finances|Éducation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanze|Formazione</t>
-  </si>
-  <si>
     <t xml:space="preserve">26.3120</t>
   </si>
   <si>
@@ -356,6 +356,36 @@
     <t xml:space="preserve">Politica nazionale|Salute</t>
   </si>
   <si>
+    <t xml:space="preserve">26.3131</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fraktion der Schweizerischen Volkspartei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Von Dänemark lernen: Bei längerfristigen Freiheitsstrafen muss die obligatorische Landesverweisung obligatorisch sein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imparare dalla Danimarca: espulsione obbligatoria in caso di pene detentive di lunga durata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die erforderlichen Gesetzesanpassungen vorzulegen, so dass für kriminelle Ausländer bei einer längerfristigen Freiheitsstrafe ab einem Jahr – unabhängig davon, ob diese unbedingt, teilbedingt oder bedingt ausfällt – in jedem Fall zwingend eine Landesverweisung angeordnet und vollzogen werden muss.&amp;nbsp;&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263131</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263131</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strafrecht|Migration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Droit pénal|Politique migratoire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diritto penale|Migrazione</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.3121</t>
   </si>
   <si>
@@ -369,36 +399,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263121</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.3131</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fraktion der Schweizerischen Volkspartei</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Von Dänemark lernen: Bei längerfristigen Freiheitsstrafen muss die obligatorische Landesverweisung obligatorisch sein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imparare dalla Danimarca: espulsione obbligatoria in caso di pene detentive di lunga durata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die erforderlichen Gesetzesanpassungen vorzulegen, so dass für kriminelle Ausländer bei einer längerfristigen Freiheitsstrafe ab einem Jahr – unabhängig davon, ob diese unbedingt, teilbedingt oder bedingt ausfällt – in jedem Fall zwingend eine Landesverweisung angeordnet und vollzogen werden muss.&amp;nbsp;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263131</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263131</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strafrecht|Migration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Droit pénal|Politique migratoire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diritto penale|Migrazione</t>
   </si>
   <si>
     <t xml:space="preserve">26.3099</t>
@@ -5251,7 +5251,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>20263228</v>
+        <v>20263323</v>
       </c>
       <c r="B6" t="s">
         <v>83</v>
@@ -5263,50 +5263,50 @@
         <v>84</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="F6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G6" t="s">
         <v>45</v>
       </c>
       <c r="H6" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="I6" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="J6" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
       <c r="K6" t="s">
         <v>49</v>
       </c>
-      <c r="L6" t="s">
-        <v>87</v>
-      </c>
-      <c r="M6"/>
+      <c r="L6"/>
+      <c r="M6" t="s">
+        <v>89</v>
+      </c>
       <c r="N6" t="s">
         <v>51</v>
       </c>
       <c r="O6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="P6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="Q6" t="s">
         <v>54</v>
       </c>
       <c r="R6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="S6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="T6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="U6" t="s">
         <v>58</v>
@@ -5315,42 +5315,42 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>20263323</v>
+        <v>20263228</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
         <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E7" t="s">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="F7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G7" t="s">
         <v>45</v>
       </c>
       <c r="H7" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="I7" t="s">
+        <v>63</v>
+      </c>
+      <c r="J7" t="s">
         <v>97</v>
-      </c>
-      <c r="J7" t="s">
-        <v>48</v>
       </c>
       <c r="K7" t="s">
         <v>49</v>
       </c>
-      <c r="L7"/>
-      <c r="M7" t="s">
+      <c r="L7" t="s">
         <v>98</v>
       </c>
+      <c r="M7"/>
       <c r="N7" t="s">
         <v>51</v>
       </c>
@@ -5443,62 +5443,60 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>20263121</v>
+        <v>20263131</v>
       </c>
       <c r="B9" t="s">
         <v>114</v>
       </c>
       <c r="C9" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" t="s">
-        <v>25</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="E9"/>
       <c r="F9" t="s">
         <v>106</v>
       </c>
       <c r="G9" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H9" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="I9" t="s">
-        <v>63</v>
+        <v>116</v>
       </c>
       <c r="J9" t="s">
-        <v>115</v>
+        <v>48</v>
       </c>
       <c r="K9" t="s">
-        <v>49</v>
-      </c>
-      <c r="L9" t="s">
-        <v>116</v>
-      </c>
-      <c r="M9"/>
+        <v>117</v>
+      </c>
+      <c r="L9"/>
+      <c r="M9" t="s">
+        <v>118</v>
+      </c>
       <c r="N9" t="s">
         <v>51</v>
       </c>
       <c r="O9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="P9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="Q9" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="R9" t="s">
-        <v>90</v>
+        <v>121</v>
       </c>
       <c r="S9" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="T9" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
       <c r="U9" t="s">
         <v>58</v>
@@ -5507,60 +5505,62 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>20263131</v>
+        <v>20263121</v>
       </c>
       <c r="B10" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="D10" t="s">
-        <v>120</v>
-      </c>
-      <c r="E10"/>
+        <v>24</v>
+      </c>
+      <c r="E10" t="s">
+        <v>25</v>
+      </c>
       <c r="F10" t="s">
         <v>106</v>
       </c>
       <c r="G10" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="H10" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="I10" t="s">
-        <v>121</v>
+        <v>63</v>
       </c>
       <c r="J10" t="s">
-        <v>48</v>
+        <v>125</v>
       </c>
       <c r="K10" t="s">
-        <v>122</v>
-      </c>
-      <c r="L10"/>
-      <c r="M10" t="s">
-        <v>123</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="L10" t="s">
+        <v>126</v>
+      </c>
+      <c r="M10"/>
       <c r="N10" t="s">
         <v>51</v>
       </c>
       <c r="O10" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P10" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="Q10" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="R10" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="S10" t="s">
-        <v>127</v>
+        <v>102</v>
       </c>
       <c r="T10" t="s">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="U10" t="s">
         <v>58</v>
@@ -5654,7 +5654,7 @@
         <v>45</v>
       </c>
       <c r="H12" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="I12" t="s">
         <v>144</v>
@@ -5895,7 +5895,7 @@
         <v>189</v>
       </c>
       <c r="E16" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F16" t="s">
         <v>190</v>
@@ -6586,13 +6586,13 @@
         <v>54</v>
       </c>
       <c r="R26" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="S26" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="T26" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="U26" t="s">
         <v>58</v>
@@ -6743,7 +6743,7 @@
         <v>346</v>
       </c>
       <c r="E29" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F29" t="s">
         <v>334</v>
@@ -6806,7 +6806,7 @@
         <v>72</v>
       </c>
       <c r="D30" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="E30" t="s">
         <v>61</v>
@@ -7016,7 +7016,7 @@
         <v>27</v>
       </c>
       <c r="H33" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="I33" t="s">
         <v>385</v>
@@ -7410,7 +7410,7 @@
         <v>45</v>
       </c>
       <c r="H39" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="I39" t="s">
         <v>458</v>
@@ -8173,7 +8173,7 @@
         <v>346</v>
       </c>
       <c r="E51" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F51" t="s">
         <v>577</v>
@@ -8344,13 +8344,13 @@
         <v>54</v>
       </c>
       <c r="R53" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="S53" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="T53" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="U53" t="s">
         <v>58</v>
@@ -8699,7 +8699,7 @@
         <v>689</v>
       </c>
       <c r="E59" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F59" t="s">
         <v>664</v>
@@ -9403,7 +9403,7 @@
         <v>346</v>
       </c>
       <c r="E70" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F70" t="s">
         <v>774</v>
@@ -10238,7 +10238,7 @@
         <v>45</v>
       </c>
       <c r="H83" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="I83" t="s">
         <v>954</v>
@@ -10436,7 +10436,7 @@
         <v>45</v>
       </c>
       <c r="H86" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="I86" t="s">
         <v>987</v>
@@ -10493,7 +10493,7 @@
         <v>995</v>
       </c>
       <c r="E87" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F87" t="s">
         <v>996</v>
@@ -10502,7 +10502,7 @@
         <v>45</v>
       </c>
       <c r="H87" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="I87" t="s">
         <v>997</v>
@@ -10620,10 +10620,10 @@
         <v>72</v>
       </c>
       <c r="D89" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="E89" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F89" t="s">
         <v>1013</v>
@@ -11143,7 +11143,7 @@
         <v>1080</v>
       </c>
       <c r="E97" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F97" t="s">
         <v>1059</v>
@@ -11280,7 +11280,7 @@
         <v>45</v>
       </c>
       <c r="H99" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="I99" t="s">
         <v>1104</v>
@@ -11337,7 +11337,7 @@
         <v>1115</v>
       </c>
       <c r="E100" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F100" t="s">
         <v>1092</v>
@@ -11667,7 +11667,7 @@
         <v>346</v>
       </c>
       <c r="E105" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F105" t="s">
         <v>1167</v>
@@ -11858,7 +11858,7 @@
         <v>130</v>
       </c>
       <c r="D108" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="E108" t="s">
         <v>61</v>
@@ -12384,7 +12384,7 @@
         <v>45</v>
       </c>
       <c r="H116" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="I116" t="s">
         <v>1285</v>
@@ -12964,7 +12964,7 @@
         <v>141</v>
       </c>
       <c r="D125" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="E125" t="s">
         <v>61</v>
@@ -13095,7 +13095,7 @@
         <v>689</v>
       </c>
       <c r="E127" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F127" t="s">
         <v>1396</v>
@@ -13368,7 +13368,7 @@
         <v>45</v>
       </c>
       <c r="H131" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="I131" t="s">
         <v>1440</v>
@@ -13557,7 +13557,7 @@
         <v>1472</v>
       </c>
       <c r="E134" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F134" t="s">
         <v>1460</v>
@@ -13621,7 +13621,7 @@
         <v>1472</v>
       </c>
       <c r="E135" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F135" t="s">
         <v>1460</v>
@@ -13818,7 +13818,7 @@
       </c>
       <c r="G138"/>
       <c r="H138" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="I138" t="s">
         <v>1508</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-04-27
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -212,7 +212,7 @@
     <t xml:space="preserve">Pour des laits et aliments infantiles sûrs en tout temps, garantir la prévention et l'information en cas de contamination</t>
   </si>
   <si>
-    <t xml:space="preserve">Titolo segue</t>
+    <t xml:space="preserve">Garantire la prevenzione e l’informazione in caso di contaminazione per far sì che il latte e gli alimenti per la prima infanzia siano sempre sicuri</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de prendre les mesures nécessaires pour assurer la sécurité de la population lors de cas de contaminations alimentaires, en particulier des laits et aliments infantiles. Il s’agit de garantir l’application des articles 26 à 29 de la loi sur les denrées alimentaires (LDAI), qui règlent les obligations des entreprises (autocontrôle, garantie de la protection de la santé, traçabilité, devoir d’assistance et obligation de renseigner). Les mesures prises visent à garantir que les cas de contamination soient communiqués rapidement aux autorités alimentaires et sanitaires ainsi qu'au public, que les rappels soient effectués dans les meilleurs délais et que les produits rappelés le soient effectivement.&lt;/p&gt;</t>
@@ -290,13 +290,13 @@
     <t xml:space="preserve">2026-03-19</t>
   </si>
   <si>
-    <t xml:space="preserve">Bahnplanung: Darf der Bundesrat die Aufträge des Parlaments ignorieren?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Planification ferroviaire : Le Conseil fédéral peut-il ignorer les mandats du Parlement ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pianificazione ferroviaria: il Consiglio federale può ignorare i mandati del Parlamento?</t>
+    <t xml:space="preserve">Bahnplanung. Darf der Bundesrat die Aufträge des Parlaments ignorieren?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planification ferroviaire. Le Conseil fédéral peut-il ignorer les mandats du Parlement ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pianificazione ferroviaria. Il Consiglio federale può ignorare i mandati del Parlamento?</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral a publié fin janvier 2026 les grandes lignes du développement des infrastructures de transport dans le cadre de Transport 45. Bien que les autorités politiques aient déjà fixé des orientations claires — notamment via l'approbation par les deux Chambres des motions &lt;strong&gt;24.4042&lt;/strong&gt; "Concept d’offre 2050" le 11 mars 2026 et &lt;strong&gt;23.3668&lt;/strong&gt; "Redondance et fiabilité de l’axe Lausanne-Genève" le 11 mars 2024 — le dossier &lt;strong&gt;"Transport 45"&lt;/strong&gt; semble n'en avoir nullement tenu compte.&amp;nbsp;&lt;/p&gt;&lt;p&gt;Dès lors, le Conseil fédéral est prié de répondre aux questions suivantes:&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Le message 2027 reposera-t-il sur ces deux motions montrant clairement la priorité d'étudier et de réaliser au plus vite la redondance sur l'arc lémanique, ainsi qu'un concept d'offre donnant la priorité aux grandes lignes nationales ? &amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Le message 2027, proposera-t-il des gains en cadence, des temps de parcours réduits, une plus grande capacité et une robustesse du réseau ferroviaire, notamment pour la Suisse romande ?&lt;/p&gt;&lt;p&gt;3. Au vu de certains nouveaux projets prévus par le T45, comment le Conseil fédéral compte-il assurer la viabilité du FIF sans prétériter les régions déjà en retard d'investissements (Jura et Arc lémanique) ?&amp;nbsp;&lt;/p&gt;&lt;p&gt;4. Le Conseil fédéral peut-il présenter l’impact territorial et économique d'un manque de développement du ferroviaire et les mesures prévues pour garantir l’équité de traitement ?&amp;nbsp;&amp;nbsp;&lt;/p&gt;&lt;p&gt;5. Dans une optique de maîtrise des dépenses publiques, le Conseil fédéral n'estime-t-il pas nécessaire de simplifier les normes de construction des CFF ?&lt;/p&gt;&lt;p&gt;6. Plus concrètement, des améliorations sont-elles prévues sur l’axe Bienne-Lausanne/Genève et la restauration définitive de liaison (à l'heure) directe Bâle/Zurich-Bienne-Genève (sans changement à Renens) ?&amp;nbsp;&lt;/p&gt;&lt;p&gt;7. Enfin, au-delà des grands chantiers, le Conseil fédéral ne pense-t-il pas prioriser des projets à haute valeur ajoutée et à faible coût, tels que la &lt;strong&gt;halte ferroviaire d'Y-Parc à Yverdon&lt;/strong&gt; ? Son investissement dérisoire pour l’OFT garantit pourtant un report modal pour des milliers d'emplois.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Si une planification technique peut balayer les décisions du Parlement, à quoi sert-il encore de siéger ?&lt;/strong&gt;&lt;/p&gt;</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-04-28
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -206,13 +206,13 @@
     <t xml:space="preserve">EDI</t>
   </si>
   <si>
-    <t xml:space="preserve">Jederzeit sichere Säuglingsnahrung: Prävention und Aufklärung im Fall einer Kontamination gewährleisten</t>
+    <t xml:space="preserve">Jederzeit sichere Säuglingsnahrung. Prävention und Aufklärung im Fall einer Kontamination gewährleisten</t>
   </si>
   <si>
     <t xml:space="preserve">Pour des laits et aliments infantiles sûrs en tout temps, garantir la prévention et l'information en cas de contamination</t>
   </si>
   <si>
-    <t xml:space="preserve">Garantire la prevenzione e l’informazione in caso di contaminazione per far sì che il latte e gli alimenti per la prima infanzia siano sempre sicuri</t>
+    <t xml:space="preserve">Garantire la prevenzione e l'informazione in caso di contaminazione per far sì che il latte e gli alimenti per la prima infanzia siano sempre sicuri</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de prendre les mesures nécessaires pour assurer la sécurité de la population lors de cas de contaminations alimentaires, en particulier des laits et aliments infantiles. Il s’agit de garantir l’application des articles 26 à 29 de la loi sur les denrées alimentaires (LDAI), qui règlent les obligations des entreprises (autocontrôle, garantie de la protection de la santé, traçabilité, devoir d’assistance et obligation de renseigner). Les mesures prises visent à garantir que les cas de contamination soient communiqués rapidement aux autorités alimentaires et sanitaires ainsi qu'au public, que les rappels soient effectués dans les meilleurs délais et que les produits rappelés le soient effectivement.&lt;/p&gt;</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-05-14
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -185,18 +185,57 @@
     <t xml:space="preserve">Economia|Questioni sociali|Media e comunicazione|Salute</t>
   </si>
   <si>
+    <t xml:space="preserve">26.3454</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ip.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stettler Thomas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UVEK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verbesserte Lebensqualität dank den Umfahrungsprojekten entlang der N18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qualité de vie améliorée grâce aux projets de contournement de la N18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Migliore qualità di vita grazie ai progetti di circonvallazione sulla N18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Fin janvier 2026, le Conseil fédéral a publié les lignes directrices de «&amp;nbsp;&lt;i&gt;Transports ’45&amp;nbsp;»&lt;/i&gt;. Selon ces derniers, les projets routiers prévus le long de la route nationale 18 entre Bâle et Delémont – à l’exception de la décharge du centre de Laufon (horizon 2055) – devraient être reportés à une période postérieure à 2055. Cette perspective suscite une vive incompréhension dans la région. Elle équivaut en effet à renoncer, pour plusieurs décennies, à une amélioration de l’accessibilité et, par conséquent, à de réelles perspectives de développement économique. Elle contredit en outre directement les résultats de l’étude de corridor N18, menée sous la conduite de l’OFROU selon les méthodes les plus récentes et soutenue par un large partenariat.&lt;/p&gt;&lt;p&gt;La N18 constitue un maillon essentiel du réseau routier national. Elle relie l’agglomération bâloise à l’Arc lémanique et dessert le Laufonnais, en plein essor, ainsi que Delémont, chef-lieu cantonal. En raison de la croissance démographique, ce tronçon devient toutefois un goulet d’étranglement, présentant l’une des charges de trafic et densités de bouchons les plus élevées du pays. La situation actuelle affecte par ailleurs fortement la qualité de vie dans les centres des localités et compromet la sécurité du trafic motorisé et cycliste. La population souffre quotidiennement des embouteillages et du trafic intense des poids lourds traversant les localités, comme en témoignent les nombreux participants aux forums de la mobilité de Laufon. Une évolution rapide du corridor apparaît dès lors indispensable.&lt;/p&gt;&lt;p&gt;Dans ce contexte, le Conseil fédéral est prié de répondre aux questions suivantes :&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Comment évalue-t-il les effets du trafic de transit – en particulier des poids lourds – sur le développement du milieu bâti ainsi que sur la qualité de séjour et d’habitation à Delémont, Laufon et Zwingen ?&lt;/li&gt;&lt;li&gt;Considère-t-il les projets de contournement Laufon–Zwingen et Delémont comme des mesures appropriées pour réduire les nuisances dans les zones urbanisées concernées ?&lt;/li&gt;&lt;li&gt;Estime-t-il nécessaires des mesures visant à améliorer la desserte des zones d’emplois à Delémont ainsi que dans le Laufonnais ?&lt;/li&gt;&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Ende Januar 2026 veröffentlichte der Bundesrat die Eckwerte von &lt;i&gt;«Verkehr ’45»&lt;/i&gt;. Die geplanten Strassenbauprojekte entlang der Nationalstrasse 18 zwischen Basel und Delsberg – mit Ausnahme der Entlastung des Zentrums von Laufen (bis 2055) – sollen auf einen Zeitpunkt nach 2055 verschoben werden. Diese Aussichten stossen in der Region auf grosses Unverständnis. Der Entscheid bedeutet nämlich, dass für mehrere Jahrzehnte auf eine Verbesserung der Erreichbarkeit und damit auf echte Perspektiven für die wirtschaftliche Entwicklung verzichtet wird. Zudem steht er in direktem Widerspruch zu den Ergebnissen der Korridorstudie N18, die unter der Leitung des ASTRA nach den neuesten Methoden durchgeführt und von einer breiten Partnerschaft unterstützt wurde.&lt;/p&gt;&lt;p&gt;Die N18 ist ein wesentlicher Abschnitt des nationalen Strassennetzes. Sie verbindet den Grossraum Basel mit der Genferseeregion und bedient das aufstrebende Laufental sowie die Kantonshauptstadt Delsberg. Aufgrund des Bevölkerungswachstums entwickelt sich dieser Abschnitt jedoch zu einem Engpass und weist eine der höchsten Verkehrsbelastungen und Staudichten des Landes auf. Die derzeitige Situation beeinträchtigt zudem erheblich die Lebensqualität in den Ortskernen und gefährdet die Sicherheit des motorisierten Verkers und des Veloverkehrs. Die Bevölkerung leidet täglich unter den Staus und dem starken Lastwagenverkehr, der durch die Ortschaften rollt, wie die zahlreichen Teilnehmer und Teilnehmerinnen der Mobilitätsforen in Laufen bezeugen. Eine rasche Weiterentwicklung des Korridors erscheint daher unerlässlich.&lt;/p&gt;&lt;p&gt;Vor diesem Hintergrund bitte ich den Bundesrat um die Beantwortung der folgenden Fragen:&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Wie bewertet er die Auswirkungen des Transitverkehrs – insbesondere des Schwerverkehrs – auf die Siedlungsentwicklung sowie auf die Lebens- und Wohnqualität in Delsberg, Laufen und Zwingen?&lt;/li&gt;&lt;li&gt;Erachtet er die Umfahrungsprojekte Laufen–Zwingen und Delsberg als geeignete Massnahmen zur Verringerung der Belastungen in den betroffenen Siedlungsgebieten?&lt;/li&gt;&lt;li&gt;Hält er Massnahmen zur Verbesserung der Verkehrsanbindung der Arbeitszonen in Delsberg sowie im Laufental für notwendig?&lt;/li&gt;&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263454</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263454</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verkehr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transports</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trasporti</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.3192</t>
   </si>
   <si>
-    <t xml:space="preserve">Ip.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Aeschi Thomas</t>
   </si>
   <si>
-    <t xml:space="preserve">UDC</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-03-18</t>
   </si>
   <si>
@@ -332,9 +371,6 @@
     <t xml:space="preserve">26.3121</t>
   </si>
   <si>
-    <t xml:space="preserve">UVEK</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dank einer leistungsfähigen Nationalstrasse 18 Kultur- und Wirtschaftsräume effektiv miteinander verbinden</t>
   </si>
   <si>
@@ -395,15 +431,6 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263069</t>
   </si>
   <si>
-    <t xml:space="preserve">Verkehr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transports</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trasporti</t>
-  </si>
-  <si>
     <t xml:space="preserve">25.4774</t>
   </si>
   <si>
@@ -444,33 +471,6 @@
   </si>
   <si>
     <t xml:space="preserve">2026-04-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.3454</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stettler Thomas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verbesserte Lebensqualität dank den Umfahrungsprojekten entlang der N18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Qualité de vie améliorée grâce aux projets de contournement de la N18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Migliore qualità di vita grazie ai progetti di circonvallazione sulla N18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Fin janvier 2026, le Conseil fédéral a publié les lignes directrices de «&amp;nbsp;&lt;i&gt;Transports ’45&amp;nbsp;»&lt;/i&gt;. Selon ces derniers, les projets routiers prévus le long de la route nationale 18 entre Bâle et Delémont – à l’exception de la décharge du centre de Laufon (horizon 2055) – devraient être reportés à une période postérieure à 2055. Cette perspective suscite une vive incompréhension dans la région. Elle équivaut en effet à renoncer, pour plusieurs décennies, à une amélioration de l’accessibilité et, par conséquent, à de réelles perspectives de développement économique. Elle contredit en outre directement les résultats de l’étude de corridor N18, menée sous la conduite de l’OFROU selon les méthodes les plus récentes et soutenue par un large partenariat.&lt;/p&gt;&lt;p&gt;La N18 constitue un maillon essentiel du réseau routier national. Elle relie l’agglomération bâloise à l’Arc lémanique et dessert le Laufonnais, en plein essor, ainsi que Delémont, chef-lieu cantonal. En raison de la croissance démographique, ce tronçon devient toutefois un goulet d’étranglement, présentant l’une des charges de trafic et densités de bouchons les plus élevées du pays. La situation actuelle affecte par ailleurs fortement la qualité de vie dans les centres des localités et compromet la sécurité du trafic motorisé et cycliste. La population souffre quotidiennement des embouteillages et du trafic intense des poids lourds traversant les localités, comme en témoignent les nombreux participants aux forums de la mobilité de Laufon. Une évolution rapide du corridor apparaît dès lors indispensable.&lt;/p&gt;&lt;p&gt;Dans ce contexte, le Conseil fédéral est prié de répondre aux questions suivantes :&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Comment évalue-t-il les effets du trafic de transit – en particulier des poids lourds – sur le développement du milieu bâti ainsi que sur la qualité de séjour et d’habitation à Delémont, Laufon et Zwingen ?&lt;/li&gt;&lt;li&gt;Considère-t-il les projets de contournement Laufon–Zwingen et Delémont comme des mesures appropriées pour réduire les nuisances dans les zones urbanisées concernées ?&lt;/li&gt;&lt;li&gt;Estime-t-il nécessaires des mesures visant à améliorer la desserte des zones d’emplois à Delémont ainsi que dans le Laufonnais ?&lt;/li&gt;&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Ende Januar 2026 veröffentlichte der Bundesrat die Eckwerte von &lt;i&gt;«Verkehr ’45»&lt;/i&gt;. Die geplanten Strassenbauprojekte entlang der Nationalstrasse 18 zwischen Basel und Delsberg – mit Ausnahme der Entlastung des Zentrums von Laufen (bis 2055) – sollen auf einen Zeitpunkt nach 2055 verschoben werden. Diese Aussichten stossen in der Region auf grosses Unverständnis. Der Entscheid bedeutet nämlich, dass für mehrere Jahrzehnte auf eine Verbesserung der Erreichbarkeit und damit auf echte Perspektiven für die wirtschaftliche Entwicklung verzichtet wird. Zudem steht er in direktem Widerspruch zu den Ergebnissen der Korridorstudie N18, die unter der Leitung des ASTRA nach den neuesten Methoden durchgeführt und von einer breiten Partnerschaft unterstützt wurde.&lt;/p&gt;&lt;p&gt;Die N18 ist ein wesentlicher Abschnitt des nationalen Strassennetzes. Sie verbindet den Grossraum Basel mit der Genferseeregion und bedient das aufstrebende Laufental sowie die Kantonshauptstadt Delsberg. Aufgrund des Bevölkerungswachstums entwickelt sich dieser Abschnitt jedoch zu einem Engpass und weist eine der höchsten Verkehrsbelastungen und Staudichten des Landes auf. Die derzeitige Situation beeinträchtigt zudem erheblich die Lebensqualität in den Ortskernen und gefährdet die Sicherheit des motorisierten Verkers und des Veloverkehrs. Die Bevölkerung leidet täglich unter den Staus und dem starken Lastwagenverkehr, der durch die Ortschaften rollt, wie die zahlreichen Teilnehmer und Teilnehmerinnen der Mobilitätsforen in Laufen bezeugen. Eine rasche Weiterentwicklung des Korridors erscheint daher unerlässlich.&lt;/p&gt;&lt;p&gt;Vor diesem Hintergrund bitte ich den Bundesrat um die Beantwortung der folgenden Fragen:&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Wie bewertet er die Auswirkungen des Transitverkehrs – insbesondere des Schwerverkehrs – auf die Siedlungsentwicklung sowie auf die Lebens- und Wohnqualität in Delsberg, Laufen und Zwingen?&lt;/li&gt;&lt;li&gt;Erachtet er die Umfahrungsprojekte Laufen–Zwingen und Delsberg als geeignete Massnahmen zur Verringerung der Belastungen in den betroffenen Siedlungsgebieten?&lt;/li&gt;&lt;li&gt;Hält er Massnahmen zur Verbesserung der Verkehrsanbindung der Arbeitszonen in Delsberg sowie im Laufental für notwendig?&lt;/li&gt;&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263454</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263454</t>
   </si>
   <si>
     <t xml:space="preserve">26.3228</t>
@@ -5230,7 +5230,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20263192</v>
+        <v>20263454</v>
       </c>
       <c r="B4" t="s">
         <v>57</v>
@@ -5245,49 +5245,49 @@
         <v>60</v>
       </c>
       <c r="F4" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="G4" t="s">
         <v>26</v>
       </c>
       <c r="H4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" t="s">
         <v>62</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>63</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>64</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>65</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>66</v>
-      </c>
-      <c r="M4" t="s">
-        <v>67</v>
       </c>
       <c r="N4" t="s">
         <v>33</v>
       </c>
       <c r="O4" t="s">
+        <v>67</v>
+      </c>
+      <c r="P4" t="s">
         <v>68</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
+        <v>53</v>
+      </c>
+      <c r="R4" t="s">
         <v>69</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="S4" t="s">
         <v>70</v>
       </c>
-      <c r="R4" t="s">
+      <c r="T4" t="s">
         <v>71</v>
-      </c>
-      <c r="S4" t="s">
-        <v>72</v>
-      </c>
-      <c r="T4" t="s">
-        <v>73</v>
       </c>
       <c r="U4" t="s">
         <v>40</v>
@@ -5296,64 +5296,64 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20263099</v>
+        <v>20263192</v>
       </c>
       <c r="B5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" t="s">
         <v>74</v>
       </c>
-      <c r="C5" t="s">
+      <c r="G5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" t="s">
         <v>75</v>
       </c>
-      <c r="D5" t="s">
+      <c r="I5" t="s">
         <v>76</v>
       </c>
-      <c r="E5" t="s">
+      <c r="J5" t="s">
         <v>77</v>
       </c>
-      <c r="F5" t="s">
+      <c r="K5" t="s">
         <v>78</v>
       </c>
-      <c r="G5" t="s">
-        <v>44</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="L5" t="s">
         <v>79</v>
       </c>
-      <c r="I5" t="s">
+      <c r="M5" t="s">
         <v>80</v>
-      </c>
-      <c r="J5" t="s">
-        <v>81</v>
-      </c>
-      <c r="K5" t="s">
-        <v>82</v>
-      </c>
-      <c r="L5" t="s">
-        <v>83</v>
-      </c>
-      <c r="M5" t="s">
-        <v>84</v>
       </c>
       <c r="N5" t="s">
         <v>33</v>
       </c>
       <c r="O5" t="s">
+        <v>81</v>
+      </c>
+      <c r="P5" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>83</v>
+      </c>
+      <c r="R5" t="s">
+        <v>84</v>
+      </c>
+      <c r="S5" t="s">
         <v>85</v>
       </c>
-      <c r="P5" t="s">
+      <c r="T5" t="s">
         <v>86</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>53</v>
-      </c>
-      <c r="R5" t="s">
-        <v>87</v>
-      </c>
-      <c r="S5" t="s">
-        <v>88</v>
-      </c>
-      <c r="T5" t="s">
-        <v>89</v>
       </c>
       <c r="U5" t="s">
         <v>40</v>
@@ -5362,28 +5362,28 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>20263120</v>
+        <v>20263099</v>
       </c>
       <c r="B6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E6" t="s">
         <v>90</v>
       </c>
-      <c r="C6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="F6" t="s">
         <v>91</v>
       </c>
-      <c r="E6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" t="s">
         <v>92</v>
-      </c>
-      <c r="G6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" t="s">
-        <v>45</v>
       </c>
       <c r="I6" t="s">
         <v>93</v>
@@ -5410,73 +5410,73 @@
         <v>99</v>
       </c>
       <c r="Q6" t="s">
+        <v>53</v>
+      </c>
+      <c r="R6" t="s">
         <v>100</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>101</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>102</v>
       </c>
-      <c r="T6" t="s">
-        <v>103</v>
-      </c>
       <c r="U6" t="s">
-        <v>104</v>
+        <v>40</v>
       </c>
       <c r="V6"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>20263121</v>
+        <v>20263120</v>
       </c>
       <c r="B7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" t="s">
         <v>105</v>
       </c>
-      <c r="C7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" t="s">
-        <v>77</v>
-      </c>
-      <c r="F7" t="s">
-        <v>92</v>
-      </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="H7" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" t="s">
         <v>106</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>107</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>108</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>109</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>110</v>
-      </c>
-      <c r="M7" t="s">
-        <v>111</v>
       </c>
       <c r="N7" t="s">
         <v>33</v>
       </c>
       <c r="O7" t="s">
+        <v>111</v>
+      </c>
+      <c r="P7" t="s">
         <v>112</v>
       </c>
-      <c r="P7" t="s">
+      <c r="Q7" t="s">
         <v>113</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>53</v>
       </c>
       <c r="R7" t="s">
         <v>114</v>
@@ -5488,100 +5488,100 @@
         <v>116</v>
       </c>
       <c r="U7" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="V7"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>20263069</v>
+        <v>20263121</v>
       </c>
       <c r="B8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C8" t="s">
         <v>58</v>
       </c>
       <c r="D8" t="s">
-        <v>118</v>
+        <v>89</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F8" t="s">
+        <v>105</v>
+      </c>
+      <c r="G8" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" t="s">
         <v>119</v>
       </c>
-      <c r="G8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H8" t="s">
-        <v>106</v>
-      </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>120</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>121</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>122</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>123</v>
-      </c>
-      <c r="M8" t="s">
-        <v>124</v>
       </c>
       <c r="N8" t="s">
         <v>33</v>
       </c>
       <c r="O8" t="s">
+        <v>124</v>
+      </c>
+      <c r="P8" t="s">
         <v>125</v>
       </c>
-      <c r="P8" t="s">
+      <c r="Q8" t="s">
+        <v>53</v>
+      </c>
+      <c r="R8" t="s">
         <v>126</v>
       </c>
-      <c r="Q8" t="s">
-        <v>36</v>
-      </c>
-      <c r="R8" t="s">
+      <c r="S8" t="s">
         <v>127</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>128</v>
       </c>
-      <c r="T8" t="s">
-        <v>129</v>
-      </c>
       <c r="U8" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="V8"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>20254774</v>
+        <v>20263069</v>
       </c>
       <c r="B9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" t="s">
         <v>130</v>
       </c>
-      <c r="C9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" t="s">
-        <v>76</v>
-      </c>
       <c r="E9" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
         <v>131</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="H9" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="I9" t="s">
         <v>132</v>
@@ -5599,98 +5599,96 @@
         <v>136</v>
       </c>
       <c r="N9" t="s">
+        <v>33</v>
+      </c>
+      <c r="O9" t="s">
         <v>137</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>138</v>
       </c>
-      <c r="P9" t="s">
-        <v>139</v>
-      </c>
       <c r="Q9" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="R9" t="s">
-        <v>140</v>
+        <v>69</v>
       </c>
       <c r="S9" t="s">
-        <v>141</v>
+        <v>70</v>
       </c>
       <c r="T9" t="s">
-        <v>142</v>
+        <v>71</v>
       </c>
       <c r="U9" t="s">
-        <v>143</v>
+        <v>117</v>
       </c>
       <c r="V9"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>20263454</v>
+        <v>20254774</v>
       </c>
       <c r="B10" t="s">
+        <v>139</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
+        <v>89</v>
+      </c>
+      <c r="E10" t="s">
+        <v>90</v>
+      </c>
+      <c r="F10" t="s">
+        <v>140</v>
+      </c>
+      <c r="G10" t="s">
+        <v>44</v>
+      </c>
+      <c r="H10" t="s">
+        <v>92</v>
+      </c>
+      <c r="I10" t="s">
+        <v>141</v>
+      </c>
+      <c r="J10" t="s">
+        <v>142</v>
+      </c>
+      <c r="K10" t="s">
+        <v>143</v>
+      </c>
+      <c r="L10" t="s">
         <v>144</v>
       </c>
-      <c r="C10" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="M10" t="s">
         <v>145</v>
       </c>
-      <c r="E10" t="s">
-        <v>60</v>
-      </c>
-      <c r="F10" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" t="s">
-        <v>106</v>
-      </c>
-      <c r="I10" t="s">
+      <c r="N10" t="s">
         <v>146</v>
       </c>
-      <c r="J10" t="s">
+      <c r="O10" t="s">
         <v>147</v>
       </c>
-      <c r="K10" t="s">
+      <c r="P10" t="s">
         <v>148</v>
-      </c>
-      <c r="L10" t="s">
-        <v>149</v>
-      </c>
-      <c r="M10" t="s">
-        <v>150</v>
-      </c>
-      <c r="N10" t="s">
-        <v>33</v>
-      </c>
-      <c r="O10" t="s">
-        <v>151</v>
-      </c>
-      <c r="P10" t="s">
-        <v>152</v>
       </c>
       <c r="Q10" t="s">
         <v>53</v>
       </c>
       <c r="R10" t="s">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="S10" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="T10" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
       <c r="U10" t="s">
-        <v>40</v>
-      </c>
-      <c r="V10" t="s">
-        <v>40</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="V10"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -5715,7 +5713,7 @@
         <v>26</v>
       </c>
       <c r="H11" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I11" t="s">
         <v>156</v>
@@ -5742,16 +5740,16 @@
         <v>163</v>
       </c>
       <c r="Q11" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R11" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="S11" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="T11" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="U11" t="s">
         <v>164</v>
@@ -5808,7 +5806,7 @@
         <v>175</v>
       </c>
       <c r="Q12" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R12" t="s">
         <v>176</v>
@@ -5839,13 +5837,13 @@
       </c>
       <c r="E13"/>
       <c r="F13" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="G13" t="s">
         <v>26</v>
       </c>
       <c r="H13" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I13" t="s">
         <v>181</v>
@@ -5872,7 +5870,7 @@
         <v>187</v>
       </c>
       <c r="Q13" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R13" t="s">
         <v>188</v>
@@ -5969,13 +5967,13 @@
         <v>207</v>
       </c>
       <c r="F15" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="G15" t="s">
         <v>26</v>
       </c>
       <c r="H15" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I15" t="s">
         <v>208</v>
@@ -6000,7 +5998,7 @@
         <v>213</v>
       </c>
       <c r="Q15" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R15" t="s">
         <v>214</v>
@@ -6033,7 +6031,7 @@
       </c>
       <c r="G16"/>
       <c r="H16" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I16" t="s">
         <v>220</v>
@@ -6059,13 +6057,13 @@
         <v>53</v>
       </c>
       <c r="R16" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="S16" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="T16" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="U16" t="s">
         <v>164</v>
@@ -6120,7 +6118,7 @@
         <v>234</v>
       </c>
       <c r="Q17" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R17" t="s">
         <v>235</v>
@@ -6184,7 +6182,7 @@
         <v>247</v>
       </c>
       <c r="Q18" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R18" t="s">
         <v>248</v>
@@ -6217,7 +6215,7 @@
         <v>253</v>
       </c>
       <c r="F19" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="G19" t="s">
         <v>26</v>
@@ -6283,13 +6281,13 @@
         <v>60</v>
       </c>
       <c r="F20" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="G20" t="s">
         <v>26</v>
       </c>
       <c r="H20" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I20" t="s">
         <v>266</v>
@@ -6316,7 +6314,7 @@
         <v>272</v>
       </c>
       <c r="Q20" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R20" t="s">
         <v>273</v>
@@ -6343,10 +6341,10 @@
         <v>23</v>
       </c>
       <c r="D21" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="E21" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F21" t="s">
         <v>277</v>
@@ -6406,13 +6404,13 @@
         <v>290</v>
       </c>
       <c r="C22" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="D22" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="E22" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F22" t="s">
         <v>277</v>
@@ -6421,7 +6419,7 @@
         <v>44</v>
       </c>
       <c r="H22" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I22" t="s">
         <v>291</v>
@@ -6478,7 +6476,7 @@
         <v>303</v>
       </c>
       <c r="E23" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F23" t="s">
         <v>304</v>
@@ -6514,7 +6512,7 @@
         <v>311</v>
       </c>
       <c r="Q23" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R23" t="s">
         <v>312</v>
@@ -6541,7 +6539,7 @@
         <v>23</v>
       </c>
       <c r="D24" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="E24" t="s">
         <v>60</v>
@@ -6580,7 +6578,7 @@
         <v>323</v>
       </c>
       <c r="Q24" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R24" t="s">
         <v>248</v>
@@ -6710,7 +6708,7 @@
         <v>343</v>
       </c>
       <c r="Q26" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R26" t="s">
         <v>344</v>
@@ -6737,7 +6735,7 @@
         <v>192</v>
       </c>
       <c r="D27" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="E27" t="s">
         <v>60</v>
@@ -6749,7 +6747,7 @@
         <v>26</v>
       </c>
       <c r="H27" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I27" t="s">
         <v>348</v>
@@ -6774,7 +6772,7 @@
         <v>353</v>
       </c>
       <c r="Q27" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R27" t="s">
         <v>188</v>
@@ -6798,7 +6796,7 @@
         <v>354</v>
       </c>
       <c r="C28" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="D28" t="s">
         <v>355</v>
@@ -6838,7 +6836,7 @@
         <v>363</v>
       </c>
       <c r="Q28" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R28" t="s">
         <v>364</v>
@@ -6904,7 +6902,7 @@
         <v>376</v>
       </c>
       <c r="Q29" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R29" t="s">
         <v>377</v>
@@ -6928,7 +6926,7 @@
         <v>380</v>
       </c>
       <c r="C30" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="D30" t="s">
         <v>381</v>
@@ -6970,16 +6968,16 @@
         <v>388</v>
       </c>
       <c r="Q30" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R30" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="S30" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="T30" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="U30" t="s">
         <v>164</v>
@@ -7009,7 +7007,7 @@
         <v>26</v>
       </c>
       <c r="H31" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I31" t="s">
         <v>390</v>
@@ -7039,13 +7037,13 @@
         <v>36</v>
       </c>
       <c r="R31" t="s">
-        <v>127</v>
+        <v>69</v>
       </c>
       <c r="S31" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="T31" t="s">
-        <v>129</v>
+        <v>71</v>
       </c>
       <c r="U31" t="s">
         <v>164</v>
@@ -7132,7 +7130,7 @@
         <v>409</v>
       </c>
       <c r="E33" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F33" t="s">
         <v>410</v>
@@ -7195,10 +7193,10 @@
         <v>58</v>
       </c>
       <c r="D34" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="E34" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F34" t="s">
         <v>419</v>
@@ -7300,7 +7298,7 @@
         <v>438</v>
       </c>
       <c r="Q35" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R35" t="s">
         <v>439</v>
@@ -7330,7 +7328,7 @@
         <v>443</v>
       </c>
       <c r="E36" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F36" t="s">
         <v>444</v>
@@ -7393,7 +7391,7 @@
         <v>456</v>
       </c>
       <c r="D37" t="s">
-        <v>145</v>
+        <v>59</v>
       </c>
       <c r="E37" t="s">
         <v>60</v>
@@ -7471,7 +7469,7 @@
         <v>26</v>
       </c>
       <c r="H38" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I38" t="s">
         <v>472</v>
@@ -7498,7 +7496,7 @@
         <v>478</v>
       </c>
       <c r="Q38" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R38" t="s">
         <v>479</v>
@@ -7592,7 +7590,7 @@
         <v>492</v>
       </c>
       <c r="E40" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F40" t="s">
         <v>471</v>
@@ -7626,7 +7624,7 @@
         <v>498</v>
       </c>
       <c r="Q40" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R40" t="s">
         <v>499</v>
@@ -7665,7 +7663,7 @@
         <v>26</v>
       </c>
       <c r="H41" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I41" t="s">
         <v>504</v>
@@ -7756,7 +7754,7 @@
         <v>522</v>
       </c>
       <c r="Q42" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R42" t="s">
         <v>523</v>
@@ -7820,7 +7818,7 @@
         <v>532</v>
       </c>
       <c r="Q43" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R43" t="s">
         <v>533</v>
@@ -7882,7 +7880,7 @@
         <v>547</v>
       </c>
       <c r="Q44" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R44"/>
       <c r="S44"/>
@@ -7915,7 +7913,7 @@
         <v>26</v>
       </c>
       <c r="H45" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I45" t="s">
         <v>551</v>
@@ -7942,7 +7940,7 @@
         <v>557</v>
       </c>
       <c r="Q45" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R45" t="s">
         <v>558</v>
@@ -7981,7 +7979,7 @@
         <v>26</v>
       </c>
       <c r="H46" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I46" t="s">
         <v>563</v>
@@ -8008,7 +8006,7 @@
         <v>569</v>
       </c>
       <c r="Q46" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R46" t="s">
         <v>570</v>
@@ -8032,13 +8030,13 @@
         <v>573</v>
       </c>
       <c r="C47" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="D47" t="s">
         <v>574</v>
       </c>
       <c r="E47" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F47" t="s">
         <v>550</v>
@@ -8074,7 +8072,7 @@
         <v>582</v>
       </c>
       <c r="Q47" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R47" t="s">
         <v>583</v>
@@ -8204,7 +8202,7 @@
         <v>606</v>
       </c>
       <c r="Q49" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R49" t="s">
         <v>607</v>
@@ -8243,7 +8241,7 @@
         <v>26</v>
       </c>
       <c r="H50" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I50" t="s">
         <v>613</v>
@@ -8273,13 +8271,13 @@
         <v>36</v>
       </c>
       <c r="R50" t="s">
-        <v>127</v>
+        <v>69</v>
       </c>
       <c r="S50" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="T50" t="s">
-        <v>129</v>
+        <v>71</v>
       </c>
       <c r="U50" t="s">
         <v>164</v>
@@ -8294,7 +8292,7 @@
         <v>620</v>
       </c>
       <c r="C51" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="D51" t="s">
         <v>621</v>
@@ -8307,7 +8305,7 @@
         <v>26</v>
       </c>
       <c r="H51" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I51" t="s">
         <v>622</v>
@@ -8334,7 +8332,7 @@
         <v>628</v>
       </c>
       <c r="Q51" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R51" t="s">
         <v>629</v>
@@ -8373,7 +8371,7 @@
         <v>26</v>
       </c>
       <c r="H52" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I52" t="s">
         <v>633</v>
@@ -8439,7 +8437,7 @@
         <v>44</v>
       </c>
       <c r="H53" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I53" t="s">
         <v>646</v>
@@ -8466,7 +8464,7 @@
         <v>652</v>
       </c>
       <c r="Q53" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R53" t="s">
         <v>558</v>
@@ -8505,7 +8503,7 @@
         <v>26</v>
       </c>
       <c r="H54" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I54" t="s">
         <v>656</v>
@@ -8532,16 +8530,16 @@
         <v>662</v>
       </c>
       <c r="Q54" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R54" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="S54" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="T54" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="U54" t="s">
         <v>164</v>
@@ -8598,7 +8596,7 @@
         <v>673</v>
       </c>
       <c r="Q55" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R55" t="s">
         <v>674</v>
@@ -8752,13 +8750,13 @@
         <v>697</v>
       </c>
       <c r="C58" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="D58" t="s">
         <v>698</v>
       </c>
       <c r="E58" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F58" t="s">
         <v>699</v>
@@ -8794,7 +8792,7 @@
         <v>707</v>
       </c>
       <c r="Q58" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R58" t="s">
         <v>708</v>
@@ -8824,7 +8822,7 @@
         <v>712</v>
       </c>
       <c r="E59" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F59" t="s">
         <v>699</v>
@@ -8860,7 +8858,7 @@
         <v>719</v>
       </c>
       <c r="Q59" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R59" t="s">
         <v>720</v>
@@ -8899,7 +8897,7 @@
         <v>26</v>
       </c>
       <c r="H60" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I60" t="s">
         <v>725</v>
@@ -8926,7 +8924,7 @@
         <v>731</v>
       </c>
       <c r="Q60" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R60" t="s">
         <v>479</v>
@@ -8956,7 +8954,7 @@
         <v>733</v>
       </c>
       <c r="E61" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F61" t="s">
         <v>734</v>
@@ -9019,10 +9017,10 @@
         <v>23</v>
       </c>
       <c r="D62" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="E62" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F62" t="s">
         <v>734</v>
@@ -9088,7 +9086,7 @@
         <v>303</v>
       </c>
       <c r="E63" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F63" t="s">
         <v>754</v>
@@ -9097,7 +9095,7 @@
         <v>44</v>
       </c>
       <c r="H63" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I63" t="s">
         <v>755</v>
@@ -9124,7 +9122,7 @@
         <v>761</v>
       </c>
       <c r="Q63" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R63" t="s">
         <v>762</v>
@@ -9190,7 +9188,7 @@
         <v>773</v>
       </c>
       <c r="Q64" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R64" t="s">
         <v>774</v>
@@ -9225,7 +9223,7 @@
       </c>
       <c r="G65"/>
       <c r="H65" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I65" t="s">
         <v>780</v>
@@ -9243,7 +9241,7 @@
         <v>784</v>
       </c>
       <c r="N65" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="O65" t="s">
         <v>785</v>
@@ -9252,7 +9250,7 @@
         <v>786</v>
       </c>
       <c r="Q65" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R65"/>
       <c r="S65"/>
@@ -9281,7 +9279,7 @@
       </c>
       <c r="G66"/>
       <c r="H66" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I66" t="s">
         <v>541</v>
@@ -9308,7 +9306,7 @@
         <v>793</v>
       </c>
       <c r="Q66" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R66"/>
       <c r="S66"/>
@@ -9339,7 +9337,7 @@
         <v>44</v>
       </c>
       <c r="H67" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I67" t="s">
         <v>797</v>
@@ -9357,7 +9355,7 @@
         <v>801</v>
       </c>
       <c r="N67" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="O67" t="s">
         <v>802</v>
@@ -9366,7 +9364,7 @@
         <v>803</v>
       </c>
       <c r="Q67" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R67" t="s">
         <v>804</v>
@@ -9405,7 +9403,7 @@
         <v>26</v>
       </c>
       <c r="H68" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I68" t="s">
         <v>809</v>
@@ -9432,7 +9430,7 @@
         <v>815</v>
       </c>
       <c r="Q68" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R68" t="s">
         <v>816</v>
@@ -9528,7 +9526,7 @@
         <v>831</v>
       </c>
       <c r="E70" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F70" t="s">
         <v>808</v>
@@ -9537,7 +9535,7 @@
         <v>26</v>
       </c>
       <c r="H70" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="I70" t="s">
         <v>832</v>
@@ -9564,7 +9562,7 @@
         <v>838</v>
       </c>
       <c r="Q70" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R70" t="s">
         <v>839</v>
@@ -9669,7 +9667,7 @@
         <v>26</v>
       </c>
       <c r="H72" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I72" t="s">
         <v>855</v>
@@ -9696,7 +9694,7 @@
         <v>861</v>
       </c>
       <c r="Q72" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R72" t="s">
         <v>862</v>
@@ -9792,7 +9790,7 @@
         <v>492</v>
       </c>
       <c r="E74" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F74" t="s">
         <v>878</v>
@@ -9801,7 +9799,7 @@
         <v>26</v>
       </c>
       <c r="H74" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I74" t="s">
         <v>879</v>
@@ -9828,7 +9826,7 @@
         <v>885</v>
       </c>
       <c r="Q74" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R74" t="s">
         <v>886</v>
@@ -9867,7 +9865,7 @@
         <v>26</v>
       </c>
       <c r="H75" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I75" t="s">
         <v>891</v>
@@ -9894,7 +9892,7 @@
         <v>897</v>
       </c>
       <c r="Q75" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R75" t="s">
         <v>898</v>
@@ -9929,7 +9927,7 @@
       </c>
       <c r="G76"/>
       <c r="H76" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I76" t="s">
         <v>903</v>
@@ -9956,7 +9954,7 @@
         <v>910</v>
       </c>
       <c r="Q76" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R76"/>
       <c r="S76"/>
@@ -9977,7 +9975,7 @@
         <v>23</v>
       </c>
       <c r="D77" t="s">
-        <v>145</v>
+        <v>59</v>
       </c>
       <c r="E77" t="s">
         <v>60</v>
@@ -10016,7 +10014,7 @@
         <v>918</v>
       </c>
       <c r="Q77" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R77" t="s">
         <v>377</v>
@@ -10055,7 +10053,7 @@
         <v>26</v>
       </c>
       <c r="H78" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I78" t="s">
         <v>922</v>
@@ -10080,7 +10078,7 @@
         <v>927</v>
       </c>
       <c r="Q78" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R78" t="s">
         <v>928</v>
@@ -10119,7 +10117,7 @@
         <v>26</v>
       </c>
       <c r="H79" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I79" t="s">
         <v>934</v>
@@ -10144,7 +10142,7 @@
         <v>939</v>
       </c>
       <c r="Q79" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R79" t="s">
         <v>816</v>
@@ -10177,7 +10175,7 @@
       </c>
       <c r="G80"/>
       <c r="H80" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I80" t="s">
         <v>942</v>
@@ -10253,7 +10251,7 @@
         <v>956</v>
       </c>
       <c r="N81" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="O81" t="s">
         <v>957</v>
@@ -10262,7 +10260,7 @@
         <v>958</v>
       </c>
       <c r="Q81" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R81" t="s">
         <v>959</v>
@@ -10297,7 +10295,7 @@
       </c>
       <c r="G82"/>
       <c r="H82" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I82" t="s">
         <v>963</v>
@@ -10324,7 +10322,7 @@
         <v>969</v>
       </c>
       <c r="Q82" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R82" t="s">
         <v>970</v>
@@ -10390,7 +10388,7 @@
         <v>981</v>
       </c>
       <c r="Q83" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R83" t="s">
         <v>982</v>
@@ -10420,7 +10418,7 @@
         <v>986</v>
       </c>
       <c r="E84" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F84" t="s">
         <v>987</v>
@@ -10456,7 +10454,7 @@
         <v>994</v>
       </c>
       <c r="Q84" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R84" t="s">
         <v>995</v>
@@ -10495,7 +10493,7 @@
         <v>26</v>
       </c>
       <c r="H85" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I85" t="s">
         <v>1000</v>
@@ -10522,7 +10520,7 @@
         <v>1006</v>
       </c>
       <c r="Q85" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R85" t="s">
         <v>640</v>
@@ -10618,7 +10616,7 @@
         <v>1020</v>
       </c>
       <c r="E87" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F87" t="s">
         <v>987</v>
@@ -10720,7 +10718,7 @@
         <v>1037</v>
       </c>
       <c r="Q88" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R88" t="s">
         <v>344</v>
@@ -10759,7 +10757,7 @@
         <v>26</v>
       </c>
       <c r="H89" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I89" t="s">
         <v>1040</v>
@@ -10787,13 +10785,13 @@
         <v>36</v>
       </c>
       <c r="R89" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="S89" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="T89" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="U89" t="s">
         <v>164</v>
@@ -10823,7 +10821,7 @@
         <v>26</v>
       </c>
       <c r="H90" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I90" t="s">
         <v>1048</v>
@@ -10853,13 +10851,13 @@
         <v>36</v>
       </c>
       <c r="R90" t="s">
-        <v>127</v>
+        <v>69</v>
       </c>
       <c r="S90" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="T90" t="s">
-        <v>129</v>
+        <v>71</v>
       </c>
       <c r="U90" t="s">
         <v>164</v>
@@ -10880,7 +10878,7 @@
         <v>1020</v>
       </c>
       <c r="E91" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F91" t="s">
         <v>1056</v>
@@ -10889,7 +10887,7 @@
         <v>26</v>
       </c>
       <c r="H91" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I91" t="s">
         <v>1057</v>
@@ -10914,7 +10912,7 @@
         <v>1062</v>
       </c>
       <c r="Q91" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R91" t="s">
         <v>479</v>
@@ -10953,7 +10951,7 @@
         <v>26</v>
       </c>
       <c r="H92" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I92" t="s">
         <v>1064</v>
@@ -10981,13 +10979,13 @@
         <v>36</v>
       </c>
       <c r="R92" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="S92" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="T92" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="U92" t="s">
         <v>164</v>
@@ -11017,7 +11015,7 @@
         <v>26</v>
       </c>
       <c r="H93" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I93" t="s">
         <v>1064</v>
@@ -11045,13 +11043,13 @@
         <v>36</v>
       </c>
       <c r="R93" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="S93" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="T93" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="U93" t="s">
         <v>164</v>
@@ -11081,7 +11079,7 @@
         <v>26</v>
       </c>
       <c r="H94" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I94" t="s">
         <v>1064</v>
@@ -11109,13 +11107,13 @@
         <v>36</v>
       </c>
       <c r="R94" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="S94" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="T94" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="U94" t="s">
         <v>164</v>
@@ -11172,7 +11170,7 @@
         <v>1088</v>
       </c>
       <c r="Q95" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R95" t="s">
         <v>1089</v>
@@ -11202,7 +11200,7 @@
         <v>574</v>
       </c>
       <c r="E96" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F96" t="s">
         <v>1093</v>
@@ -11238,7 +11236,7 @@
         <v>1100</v>
       </c>
       <c r="Q96" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R96" t="s">
         <v>37</v>
@@ -11277,7 +11275,7 @@
         <v>26</v>
       </c>
       <c r="H97" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I97" t="s">
         <v>1103</v>
@@ -11304,7 +11302,7 @@
         <v>1109</v>
       </c>
       <c r="Q97" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R97" t="s">
         <v>1110</v>
@@ -11370,7 +11368,7 @@
         <v>1121</v>
       </c>
       <c r="Q98" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R98" t="s">
         <v>1122</v>
@@ -11423,7 +11421,7 @@
         <v>1131</v>
       </c>
       <c r="N99" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="O99" t="s">
         <v>1132</v>
@@ -11432,7 +11430,7 @@
         <v>1133</v>
       </c>
       <c r="Q99" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R99" t="s">
         <v>1134</v>
@@ -11462,7 +11460,7 @@
         <v>409</v>
       </c>
       <c r="E100" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F100" t="s">
         <v>1126</v>
@@ -11498,7 +11496,7 @@
         <v>1144</v>
       </c>
       <c r="Q100" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R100" t="s">
         <v>1145</v>
@@ -11564,7 +11562,7 @@
         <v>1156</v>
       </c>
       <c r="Q101" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R101" t="s">
         <v>1157</v>
@@ -11669,7 +11667,7 @@
         <v>26</v>
       </c>
       <c r="H103" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I103" t="s">
         <v>1170</v>
@@ -11696,7 +11694,7 @@
         <v>1176</v>
       </c>
       <c r="Q103" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R103" t="s">
         <v>1177</v>
@@ -11762,7 +11760,7 @@
         <v>1188</v>
       </c>
       <c r="Q104" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R104" t="s">
         <v>1189</v>
@@ -11789,7 +11787,7 @@
         <v>58</v>
       </c>
       <c r="D105" t="s">
-        <v>145</v>
+        <v>59</v>
       </c>
       <c r="E105" t="s">
         <v>60</v>
@@ -11801,7 +11799,7 @@
         <v>26</v>
       </c>
       <c r="H105" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I105" t="s">
         <v>1194</v>
@@ -11828,16 +11826,16 @@
         <v>1200</v>
       </c>
       <c r="Q105" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R105" t="s">
-        <v>127</v>
+        <v>69</v>
       </c>
       <c r="S105" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="T105" t="s">
-        <v>129</v>
+        <v>71</v>
       </c>
       <c r="U105" t="s">
         <v>164</v>
@@ -11958,7 +11956,7 @@
         <v>1218</v>
       </c>
       <c r="Q107" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R107" t="s">
         <v>685</v>
@@ -11997,7 +11995,7 @@
         <v>26</v>
       </c>
       <c r="H108" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I108" t="s">
         <v>1221</v>
@@ -12022,7 +12020,7 @@
         <v>1226</v>
       </c>
       <c r="Q108" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R108" t="s">
         <v>1227</v>
@@ -12046,7 +12044,7 @@
         <v>1230</v>
       </c>
       <c r="C109" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="D109" t="s">
         <v>154</v>
@@ -12061,7 +12059,7 @@
         <v>26</v>
       </c>
       <c r="H109" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I109" t="s">
         <v>1232</v>
@@ -12121,7 +12119,7 @@
       </c>
       <c r="G110"/>
       <c r="H110" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I110" t="s">
         <v>1241</v>
@@ -12179,7 +12177,7 @@
       </c>
       <c r="G111"/>
       <c r="H111" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I111" t="s">
         <v>1252</v>
@@ -12206,7 +12204,7 @@
         <v>1258</v>
       </c>
       <c r="Q111" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R111" t="s">
         <v>1259</v>
@@ -12245,7 +12243,7 @@
         <v>26</v>
       </c>
       <c r="H112" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I112" t="s">
         <v>1265</v>
@@ -12377,7 +12375,7 @@
         <v>44</v>
       </c>
       <c r="H114" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I114" t="s">
         <v>1289</v>
@@ -12404,7 +12402,7 @@
         <v>1295</v>
       </c>
       <c r="Q114" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R114" t="s">
         <v>640</v>
@@ -12428,13 +12426,13 @@
         <v>1296</v>
       </c>
       <c r="C115" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="D115" t="s">
         <v>303</v>
       </c>
       <c r="E115" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F115" t="s">
         <v>1297</v>
@@ -12470,7 +12468,7 @@
         <v>1304</v>
       </c>
       <c r="Q115" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R115" t="s">
         <v>1134</v>
@@ -12500,7 +12498,7 @@
         <v>1306</v>
       </c>
       <c r="E116" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F116" t="s">
         <v>1297</v>
@@ -12509,7 +12507,7 @@
         <v>26</v>
       </c>
       <c r="H116" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I116" t="s">
         <v>1307</v>
@@ -12602,7 +12600,7 @@
         <v>1326</v>
       </c>
       <c r="Q117" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R117" t="s">
         <v>1327</v>
@@ -12641,7 +12639,7 @@
         <v>26</v>
       </c>
       <c r="H118" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I118" t="s">
         <v>1331</v>
@@ -12668,7 +12666,7 @@
         <v>1337</v>
       </c>
       <c r="Q118" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R118" t="s">
         <v>1338</v>
@@ -12698,7 +12696,7 @@
         <v>1306</v>
       </c>
       <c r="E119" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F119" t="s">
         <v>1297</v>
@@ -12734,7 +12732,7 @@
         <v>1348</v>
       </c>
       <c r="Q119" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R119" t="s">
         <v>1349</v>
@@ -12800,7 +12798,7 @@
         <v>1359</v>
       </c>
       <c r="Q120" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R120" t="s">
         <v>1360</v>
@@ -12830,7 +12828,7 @@
         <v>1364</v>
       </c>
       <c r="E121" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F121" t="s">
         <v>1365</v>
@@ -12866,7 +12864,7 @@
         <v>1372</v>
       </c>
       <c r="Q121" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R121" t="s">
         <v>685</v>
@@ -12893,7 +12891,7 @@
         <v>58</v>
       </c>
       <c r="D122" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="E122" t="s">
         <v>60</v>
@@ -12932,7 +12930,7 @@
         <v>1381</v>
       </c>
       <c r="Q122" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R122" t="s">
         <v>261</v>
@@ -12998,7 +12996,7 @@
         <v>1391</v>
       </c>
       <c r="Q123" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R123" t="s">
         <v>607</v>
@@ -13022,7 +13020,7 @@
         <v>1392</v>
       </c>
       <c r="C124" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="D124" t="s">
         <v>1393</v>
@@ -13064,7 +13062,7 @@
         <v>1401</v>
       </c>
       <c r="Q124" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R124" t="s">
         <v>1157</v>
@@ -13103,7 +13101,7 @@
         <v>26</v>
       </c>
       <c r="H125" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I125" t="s">
         <v>1403</v>
@@ -13131,13 +13129,13 @@
         <v>36</v>
       </c>
       <c r="R125" t="s">
-        <v>127</v>
+        <v>69</v>
       </c>
       <c r="S125" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="T125" t="s">
-        <v>129</v>
+        <v>71</v>
       </c>
       <c r="U125" t="s">
         <v>164</v>
@@ -13167,7 +13165,7 @@
         <v>26</v>
       </c>
       <c r="H126" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I126" t="s">
         <v>1411</v>
@@ -13192,16 +13190,16 @@
         <v>1416</v>
       </c>
       <c r="Q126" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R126" t="s">
-        <v>127</v>
+        <v>69</v>
       </c>
       <c r="S126" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="T126" t="s">
-        <v>129</v>
+        <v>71</v>
       </c>
       <c r="U126" t="s">
         <v>164</v>
@@ -13295,7 +13293,7 @@
         <v>26</v>
       </c>
       <c r="H128" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I128" t="s">
         <v>1432</v>
@@ -13322,7 +13320,7 @@
         <v>1438</v>
       </c>
       <c r="Q128" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R128" t="s">
         <v>1439</v>
@@ -13388,7 +13386,7 @@
         <v>1449</v>
       </c>
       <c r="Q129" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R129" t="s">
         <v>1450</v>
@@ -13454,7 +13452,7 @@
         <v>1462</v>
       </c>
       <c r="Q130" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R130" t="s">
         <v>1463</v>
@@ -13520,7 +13518,7 @@
         <v>1468</v>
       </c>
       <c r="Q131" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R131" t="s">
         <v>1469</v>
@@ -13586,7 +13584,7 @@
         <v>1481</v>
       </c>
       <c r="Q132" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R132" t="s">
         <v>479</v>
@@ -13613,10 +13611,10 @@
         <v>58</v>
       </c>
       <c r="D133" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="E133" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F133" t="s">
         <v>1483</v>
@@ -13625,7 +13623,7 @@
         <v>44</v>
       </c>
       <c r="H133" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I133" t="s">
         <v>1484</v>
@@ -13652,7 +13650,7 @@
         <v>1490</v>
       </c>
       <c r="Q133" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R133" t="s">
         <v>1491</v>
@@ -13691,7 +13689,7 @@
         <v>26</v>
       </c>
       <c r="H134" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I134" t="s">
         <v>1496</v>
@@ -13718,7 +13716,7 @@
         <v>1502</v>
       </c>
       <c r="Q134" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R134" t="s">
         <v>1503</v>
@@ -13757,7 +13755,7 @@
         <v>26</v>
       </c>
       <c r="H135" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I135" t="s">
         <v>1508</v>
@@ -13782,7 +13780,7 @@
         <v>1513</v>
       </c>
       <c r="Q135" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R135" t="s">
         <v>1503</v>
@@ -13821,7 +13819,7 @@
         <v>26</v>
       </c>
       <c r="H136" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I136" t="s">
         <v>1515</v>
@@ -13885,7 +13883,7 @@
         <v>26</v>
       </c>
       <c r="H137" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="I137" t="s">
         <v>1524</v>
@@ -13940,7 +13938,7 @@
         <v>1306</v>
       </c>
       <c r="E138" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F138" t="s">
         <v>1531</v>
@@ -13974,7 +13972,7 @@
         <v>1537</v>
       </c>
       <c r="Q138" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="R138" t="s">
         <v>1538</v>
@@ -14036,7 +14034,7 @@
         <v>1549</v>
       </c>
       <c r="Q139" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="R139" t="s">
         <v>1550</v>

</xml_diff>